<commit_message>
AV JAVA ...... 06Jun2024
</commit_message>
<xml_diff>
--- a/03 Assessments/NOTAS AV - POO Java - 2024.1 Wyden UniRuy.xlsx
+++ b/03 Assessments/NOTAS AV - POO Java - 2024.1 Wyden UniRuy.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\heleno\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\YduqsArea1\16 WydenArea1 Desenvolvimento de Software Java\03 Assessments\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E10A0C11-FD04-4FC8-8CAD-C3415D57BC54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D545160-FE72-466C-BD1D-E6807874B7D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{413AB662-3705-4BE9-8AD4-FDF0F3F54212}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="60">
   <si>
     <t>PBL</t>
   </si>
@@ -207,13 +207,25 @@
   </si>
   <si>
     <t>Matheus de jesus menezes tavares </t>
+  </si>
+  <si>
+    <t>GitHub - Brunosm11/wayfit: Projeto acadêmico em java para controle de alunos em uma academia.</t>
+  </si>
+  <si>
+    <t>dia 12/06 - postagem</t>
+  </si>
+  <si>
+    <t>Desistiu</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+  </numFmts>
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -248,8 +260,15 @@
       <name val="Tahoma"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -268,6 +287,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="15">
     <border>
@@ -466,11 +491,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -496,65 +522,61 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="3" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="4" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="6" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="2" fillId="4" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="2" fillId="3" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="2" fillId="3" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="8" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="2" fillId="0" borderId="9" xfId="2" applyFont="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Vírgula" xfId="2" builtinId="3"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -900,14 +922,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="22" t="s">
         <v>48</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
     </row>
     <row r="2" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
@@ -933,18 +955,25 @@
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="11" t="s">
         <v>12</v>
       </c>
       <c r="B3" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="14" t="s">
-        <v>3</v>
-      </c>
-      <c r="D3" s="15"/>
-      <c r="E3" s="15"/>
-      <c r="F3" s="16"/>
+      <c r="C3" s="12" t="s">
+        <v>3</v>
+      </c>
+      <c r="D3" s="26">
+        <v>3</v>
+      </c>
+      <c r="E3" s="26">
+        <v>5</v>
+      </c>
+      <c r="F3" s="27">
+        <f>D3+E3</f>
+        <v>8</v>
+      </c>
       <c r="G3" s="1">
         <v>2</v>
       </c>
@@ -953,7 +982,7 @@
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="17" t="s">
+      <c r="A4" s="13" t="s">
         <v>14</v>
       </c>
       <c r="B4" s="6" t="s">
@@ -962,42 +991,76 @@
       <c r="C4" s="10">
         <v>0.5</v>
       </c>
-      <c r="D4" s="12"/>
-      <c r="E4" s="12"/>
-      <c r="F4" s="18"/>
+      <c r="D4" s="28">
+        <v>3</v>
+      </c>
+      <c r="E4" s="28">
+        <v>5.5</v>
+      </c>
+      <c r="F4" s="29">
+        <f t="shared" ref="F4:F22" si="0">D4+E4</f>
+        <v>8.5</v>
+      </c>
+      <c r="G4" s="1">
+        <v>9</v>
+      </c>
+      <c r="H4" s="8" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="35" t="s">
+      <c r="A5" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="31" t="s">
+      <c r="B5" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="32" t="s">
-        <v>3</v>
-      </c>
-      <c r="D5" s="33"/>
-      <c r="E5" s="12"/>
-      <c r="F5" s="18"/>
-      <c r="G5" s="34"/>
+      <c r="C5" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="D5" s="28">
+        <v>3</v>
+      </c>
+      <c r="E5" s="28">
+        <v>5.5</v>
+      </c>
+      <c r="F5" s="29">
+        <f t="shared" si="0"/>
+        <v>8.5</v>
+      </c>
+      <c r="G5" s="1">
+        <v>9</v>
+      </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" s="17" t="s">
+      <c r="A6" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="24" t="s">
+      <c r="B6" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="25" t="s">
-        <v>3</v>
-      </c>
-      <c r="D6" s="27"/>
-      <c r="E6" s="12"/>
-      <c r="F6" s="18"/>
-      <c r="G6" s="26"/>
+      <c r="C6" s="24" t="s">
+        <v>3</v>
+      </c>
+      <c r="D6" s="30">
+        <v>0</v>
+      </c>
+      <c r="E6" s="28">
+        <v>0</v>
+      </c>
+      <c r="F6" s="29">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G6" s="25">
+        <v>10</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7" s="17" t="s">
+      <c r="A7" s="13" t="s">
         <v>18</v>
       </c>
       <c r="B7" s="6" t="s">
@@ -1006,29 +1069,49 @@
       <c r="C7" s="10">
         <v>0.7</v>
       </c>
-      <c r="D7" s="12"/>
-      <c r="E7" s="12"/>
-      <c r="F7" s="18"/>
+      <c r="D7" s="28">
+        <v>3</v>
+      </c>
+      <c r="E7" s="28">
+        <v>7</v>
+      </c>
+      <c r="F7" s="29">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
       <c r="G7" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8" s="17" t="s">
+      <c r="A8" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="C8" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="D8" s="12"/>
-      <c r="E8" s="12"/>
-      <c r="F8" s="18"/>
+      <c r="C8" s="24" t="s">
+        <v>3</v>
+      </c>
+      <c r="D8" s="30">
+        <v>0</v>
+      </c>
+      <c r="E8" s="28">
+        <v>0</v>
+      </c>
+      <c r="F8" s="29">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G8" s="25">
+        <v>11</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A9" s="17" t="s">
+      <c r="A9" s="13" t="s">
         <v>22</v>
       </c>
       <c r="B9" s="6" t="s">
@@ -1037,13 +1120,23 @@
       <c r="C9" s="10">
         <v>0.6</v>
       </c>
-      <c r="D9" s="12"/>
-      <c r="E9" s="12"/>
-      <c r="F9" s="18"/>
+      <c r="D9" s="28">
+        <v>3</v>
+      </c>
+      <c r="E9" s="28">
+        <v>7</v>
+      </c>
+      <c r="F9" s="29">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
+      <c r="G9" s="1">
+        <v>1</v>
+      </c>
       <c r="H9" s="8"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A10" s="17" t="s">
+      <c r="A10" s="13" t="s">
         <v>24</v>
       </c>
       <c r="B10" s="6" t="s">
@@ -1052,9 +1145,16 @@
       <c r="C10" s="10">
         <v>0.9</v>
       </c>
-      <c r="D10" s="12"/>
-      <c r="E10" s="12"/>
-      <c r="F10" s="18"/>
+      <c r="D10" s="28">
+        <v>3</v>
+      </c>
+      <c r="E10" s="28">
+        <v>7</v>
+      </c>
+      <c r="F10" s="29">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
       <c r="G10" s="1">
         <v>4</v>
       </c>
@@ -1063,22 +1163,31 @@
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A11" s="17" t="s">
+      <c r="A11" s="13" t="s">
         <v>26</v>
       </c>
-      <c r="B11" s="24" t="s">
+      <c r="B11" s="16" t="s">
         <v>27</v>
       </c>
-      <c r="C11" s="25" t="s">
-        <v>3</v>
-      </c>
-      <c r="D11" s="27"/>
-      <c r="E11" s="12"/>
-      <c r="F11" s="18"/>
-      <c r="G11" s="26"/>
+      <c r="C11" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="D11" s="31">
+        <v>0</v>
+      </c>
+      <c r="E11" s="28">
+        <v>0</v>
+      </c>
+      <c r="F11" s="29">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G11" s="18" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A12" s="35" t="s">
+      <c r="A12" s="21" t="s">
         <v>8</v>
       </c>
       <c r="B12" s="6" t="s">
@@ -1087,9 +1196,16 @@
       <c r="C12" s="10">
         <v>0</v>
       </c>
-      <c r="D12" s="11"/>
-      <c r="E12" s="12"/>
-      <c r="F12" s="18"/>
+      <c r="D12" s="28">
+        <v>3</v>
+      </c>
+      <c r="E12" s="28">
+        <v>7</v>
+      </c>
+      <c r="F12" s="29">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
       <c r="G12" s="1">
         <v>6</v>
       </c>
@@ -1098,7 +1214,7 @@
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A13" s="17" t="s">
+      <c r="A13" s="13" t="s">
         <v>28</v>
       </c>
       <c r="B13" s="6" t="s">
@@ -1107,15 +1223,22 @@
       <c r="C13" s="10">
         <v>0.6</v>
       </c>
-      <c r="D13" s="12"/>
-      <c r="E13" s="12"/>
-      <c r="F13" s="18"/>
+      <c r="D13" s="28">
+        <v>3</v>
+      </c>
+      <c r="E13" s="28">
+        <v>7</v>
+      </c>
+      <c r="F13" s="29">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
       <c r="G13" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A14" s="17" t="s">
+      <c r="A14" s="13" t="s">
         <v>30</v>
       </c>
       <c r="B14" s="6" t="s">
@@ -1124,15 +1247,22 @@
       <c r="C14" s="10">
         <v>0.7</v>
       </c>
-      <c r="D14" s="12"/>
-      <c r="E14" s="12"/>
-      <c r="F14" s="18"/>
+      <c r="D14" s="28">
+        <v>3</v>
+      </c>
+      <c r="E14" s="28">
+        <v>7</v>
+      </c>
+      <c r="F14" s="29">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
       <c r="G14" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A15" s="17" t="s">
+      <c r="A15" s="13" t="s">
         <v>32</v>
       </c>
       <c r="B15" s="6" t="s">
@@ -1141,15 +1271,22 @@
       <c r="C15" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="D15" s="12"/>
-      <c r="E15" s="12"/>
-      <c r="F15" s="18"/>
+      <c r="D15" s="28">
+        <v>3</v>
+      </c>
+      <c r="E15" s="28">
+        <v>7</v>
+      </c>
+      <c r="F15" s="29">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
       <c r="G15" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A16" s="17" t="s">
+      <c r="A16" s="13" t="s">
         <v>34</v>
       </c>
       <c r="B16" s="6" t="s">
@@ -1158,15 +1295,22 @@
       <c r="C16" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="D16" s="12"/>
-      <c r="E16" s="12"/>
-      <c r="F16" s="18"/>
+      <c r="D16" s="28">
+        <v>3</v>
+      </c>
+      <c r="E16" s="28">
+        <v>5</v>
+      </c>
+      <c r="F16" s="29">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
       <c r="G16" s="1">
         <v>2</v>
       </c>
     </row>
     <row r="17" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A17" s="35" t="s">
+      <c r="A17" s="21" t="s">
         <v>10</v>
       </c>
       <c r="B17" s="6" t="s">
@@ -1175,9 +1319,16 @@
       <c r="C17" s="10">
         <v>0.5</v>
       </c>
-      <c r="D17" s="11"/>
-      <c r="E17" s="12"/>
-      <c r="F17" s="18"/>
+      <c r="D17" s="28">
+        <v>3</v>
+      </c>
+      <c r="E17" s="28">
+        <v>7</v>
+      </c>
+      <c r="F17" s="29">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
       <c r="G17" s="1">
         <v>7</v>
       </c>
@@ -1186,7 +1337,7 @@
       </c>
     </row>
     <row r="18" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A18" s="17" t="s">
+      <c r="A18" s="13" t="s">
         <v>36</v>
       </c>
       <c r="B18" s="6" t="s">
@@ -1195,9 +1346,16 @@
       <c r="C18" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="D18" s="12"/>
-      <c r="E18" s="12"/>
-      <c r="F18" s="18"/>
+      <c r="D18" s="28">
+        <v>3</v>
+      </c>
+      <c r="E18" s="28">
+        <v>4</v>
+      </c>
+      <c r="F18" s="29">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
       <c r="G18" s="1">
         <v>5</v>
       </c>
@@ -1209,26 +1367,34 @@
       </c>
     </row>
     <row r="19" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A19" s="17" t="s">
+      <c r="A19" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="B19" s="6" t="s">
+      <c r="B19" s="23" t="s">
         <v>39</v>
       </c>
-      <c r="C19" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="D19" s="12">
-        <v>0</v>
-      </c>
-      <c r="E19" s="12"/>
-      <c r="F19" s="18"/>
-      <c r="G19" s="1">
+      <c r="C19" s="24" t="s">
+        <v>3</v>
+      </c>
+      <c r="D19" s="30">
+        <v>0</v>
+      </c>
+      <c r="E19" s="28">
+        <v>0</v>
+      </c>
+      <c r="F19" s="29">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G19" s="25">
         <v>8</v>
       </c>
+      <c r="H19" s="1" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A20" s="17" t="s">
+      <c r="A20" s="13" t="s">
         <v>40</v>
       </c>
       <c r="B20" s="6" t="s">
@@ -1237,9 +1403,16 @@
       <c r="C20" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="D20" s="12"/>
-      <c r="E20" s="12"/>
-      <c r="F20" s="18"/>
+      <c r="D20" s="28">
+        <v>3</v>
+      </c>
+      <c r="E20" s="28">
+        <v>7</v>
+      </c>
+      <c r="F20" s="29">
+        <f t="shared" si="0"/>
+        <v>10</v>
+      </c>
       <c r="G20" s="1">
         <v>3</v>
       </c>
@@ -1248,33 +1421,52 @@
       </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="A21" s="17" t="s">
+      <c r="A21" s="13" t="s">
         <v>42</v>
       </c>
-      <c r="B21" s="6" t="s">
+      <c r="B21" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="C21" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="D21" s="12"/>
-      <c r="E21" s="12"/>
-      <c r="F21" s="18"/>
+      <c r="C21" s="17" t="s">
+        <v>3</v>
+      </c>
+      <c r="D21" s="31">
+        <v>0</v>
+      </c>
+      <c r="E21" s="28">
+        <v>0</v>
+      </c>
+      <c r="F21" s="29">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G21" s="18" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="22" spans="1:15" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A22" s="19" t="s">
+      <c r="A22" s="14" t="s">
         <v>44</v>
       </c>
-      <c r="B22" s="28" t="s">
+      <c r="B22" s="19" t="s">
         <v>45</v>
       </c>
-      <c r="C22" s="29" t="s">
-        <v>3</v>
-      </c>
-      <c r="D22" s="30"/>
-      <c r="E22" s="20"/>
-      <c r="F22" s="21"/>
-      <c r="G22" s="26"/>
+      <c r="C22" s="20" t="s">
+        <v>3</v>
+      </c>
+      <c r="D22" s="32">
+        <v>0</v>
+      </c>
+      <c r="E22" s="33">
+        <v>0</v>
+      </c>
+      <c r="F22" s="34">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G22" s="18" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="23" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A23"/>
@@ -1283,7 +1475,7 @@
     </row>
     <row r="24" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A24"/>
-      <c r="B24" s="22" t="s">
+      <c r="B24" s="15" t="s">
         <v>47</v>
       </c>
       <c r="C24"/>
@@ -1312,6 +1504,7 @@
     <hyperlink ref="H10" r:id="rId4" display="https://github.com/Gusrrocha/Librell" xr:uid="{99BE23B7-8007-43B6-9405-E2F48F9D4382}"/>
     <hyperlink ref="H12" r:id="rId5" display="https://github.com/IgorRdrigues/Projeto-Java" xr:uid="{6411B9AA-E50B-479A-B839-F898EC0ECF1F}"/>
     <hyperlink ref="H17" r:id="rId6" display="https://github.com/NotKing22/Javaweb-project" xr:uid="{51423599-3084-441B-9700-DDD603589AFF}"/>
+    <hyperlink ref="H4" r:id="rId7" display="https://github.com/Brunosm11/wayfit" xr:uid="{EC5ED2FC-232A-4FD2-9CA7-821BDDB52568}"/>
   </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>

<commit_message>
relatório Java POO ...... 08Jun2024
</commit_message>
<xml_diff>
--- a/03 Assessments/NOTAS AV - POO Java - 2024.1 Wyden UniRuy.xlsx
+++ b/03 Assessments/NOTAS AV - POO Java - 2024.1 Wyden UniRuy.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\YduqsArea1\16 WydenArea1 Desenvolvimento de Software Java\03 Assessments\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D545160-FE72-466C-BD1D-E6807874B7D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5F17939-3225-4C76-98B5-9D2F49E6FC2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{413AB662-3705-4BE9-8AD4-FDF0F3F54212}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="61">
   <si>
     <t>PBL</t>
   </si>
@@ -216,6 +216,9 @@
   </si>
   <si>
     <t>Desistiu</t>
+  </si>
+  <si>
+    <t>GitHub - jairocket/find-your-home: Atividade acadêmica para avaliação da disciplina Programação Orientada a Objetos com Java</t>
   </si>
 </sst>
 </file>
@@ -553,9 +556,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -572,6 +572,9 @@
     <xf numFmtId="43" fontId="2" fillId="3" borderId="8" xfId="2" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="43" fontId="2" fillId="0" borderId="8" xfId="2" applyFont="1" applyBorder="1"/>
     <xf numFmtId="43" fontId="2" fillId="0" borderId="9" xfId="2" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
@@ -922,14 +925,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="34" t="s">
         <v>48</v>
       </c>
-      <c r="B1" s="22"/>
-      <c r="C1" s="22"/>
-      <c r="D1" s="22"/>
-      <c r="E1" s="22"/>
-      <c r="F1" s="22"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
     </row>
     <row r="2" spans="1:8" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
@@ -964,13 +967,13 @@
       <c r="C3" s="12" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="26">
-        <v>3</v>
-      </c>
-      <c r="E3" s="26">
+      <c r="D3" s="25">
+        <v>3</v>
+      </c>
+      <c r="E3" s="25">
         <v>5</v>
       </c>
-      <c r="F3" s="27">
+      <c r="F3" s="26">
         <f>D3+E3</f>
         <v>8</v>
       </c>
@@ -991,13 +994,13 @@
       <c r="C4" s="10">
         <v>0.5</v>
       </c>
-      <c r="D4" s="28">
-        <v>3</v>
-      </c>
-      <c r="E4" s="28">
+      <c r="D4" s="27">
+        <v>3</v>
+      </c>
+      <c r="E4" s="27">
         <v>5.5</v>
       </c>
-      <c r="F4" s="29">
+      <c r="F4" s="28">
         <f t="shared" ref="F4:F22" si="0">D4+E4</f>
         <v>8.5</v>
       </c>
@@ -1018,13 +1021,13 @@
       <c r="C5" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="28">
-        <v>3</v>
-      </c>
-      <c r="E5" s="28">
+      <c r="D5" s="27">
+        <v>3</v>
+      </c>
+      <c r="E5" s="27">
         <v>5.5</v>
       </c>
-      <c r="F5" s="29">
+      <c r="F5" s="28">
         <f t="shared" si="0"/>
         <v>8.5</v>
       </c>
@@ -1036,23 +1039,23 @@
       <c r="A6" s="13" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="23" t="s">
+      <c r="B6" s="22" t="s">
         <v>17</v>
       </c>
-      <c r="C6" s="24" t="s">
-        <v>3</v>
-      </c>
-      <c r="D6" s="30">
-        <v>0</v>
-      </c>
-      <c r="E6" s="28">
-        <v>0</v>
-      </c>
-      <c r="F6" s="29">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G6" s="25">
+      <c r="C6" s="23" t="s">
+        <v>3</v>
+      </c>
+      <c r="D6" s="29">
+        <v>0</v>
+      </c>
+      <c r="E6" s="27">
+        <v>0</v>
+      </c>
+      <c r="F6" s="28">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G6" s="24">
         <v>10</v>
       </c>
       <c r="H6" s="1" t="s">
@@ -1069,13 +1072,13 @@
       <c r="C7" s="10">
         <v>0.7</v>
       </c>
-      <c r="D7" s="28">
-        <v>3</v>
-      </c>
-      <c r="E7" s="28">
+      <c r="D7" s="27">
+        <v>3</v>
+      </c>
+      <c r="E7" s="27">
         <v>7</v>
       </c>
-      <c r="F7" s="29">
+      <c r="F7" s="28">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
@@ -1087,23 +1090,23 @@
       <c r="A8" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="B8" s="23" t="s">
+      <c r="B8" s="22" t="s">
         <v>21</v>
       </c>
-      <c r="C8" s="24" t="s">
-        <v>3</v>
-      </c>
-      <c r="D8" s="30">
-        <v>0</v>
-      </c>
-      <c r="E8" s="28">
-        <v>0</v>
-      </c>
-      <c r="F8" s="29">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G8" s="25">
+      <c r="C8" s="23" t="s">
+        <v>3</v>
+      </c>
+      <c r="D8" s="29">
+        <v>0</v>
+      </c>
+      <c r="E8" s="27">
+        <v>0</v>
+      </c>
+      <c r="F8" s="28">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G8" s="24">
         <v>11</v>
       </c>
       <c r="H8" s="1" t="s">
@@ -1120,13 +1123,13 @@
       <c r="C9" s="10">
         <v>0.6</v>
       </c>
-      <c r="D9" s="28">
-        <v>3</v>
-      </c>
-      <c r="E9" s="28">
+      <c r="D9" s="27">
+        <v>3</v>
+      </c>
+      <c r="E9" s="27">
         <v>7</v>
       </c>
-      <c r="F9" s="29">
+      <c r="F9" s="28">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
@@ -1145,13 +1148,13 @@
       <c r="C10" s="10">
         <v>0.9</v>
       </c>
-      <c r="D10" s="28">
-        <v>3</v>
-      </c>
-      <c r="E10" s="28">
+      <c r="D10" s="27">
+        <v>3</v>
+      </c>
+      <c r="E10" s="27">
         <v>7</v>
       </c>
-      <c r="F10" s="29">
+      <c r="F10" s="28">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
@@ -1172,13 +1175,13 @@
       <c r="C11" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="D11" s="31">
-        <v>0</v>
-      </c>
-      <c r="E11" s="28">
-        <v>0</v>
-      </c>
-      <c r="F11" s="29">
+      <c r="D11" s="30">
+        <v>0</v>
+      </c>
+      <c r="E11" s="27">
+        <v>0</v>
+      </c>
+      <c r="F11" s="28">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -1196,13 +1199,13 @@
       <c r="C12" s="10">
         <v>0</v>
       </c>
-      <c r="D12" s="28">
-        <v>3</v>
-      </c>
-      <c r="E12" s="28">
+      <c r="D12" s="27">
+        <v>3</v>
+      </c>
+      <c r="E12" s="27">
         <v>7</v>
       </c>
-      <c r="F12" s="29">
+      <c r="F12" s="28">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
@@ -1223,13 +1226,13 @@
       <c r="C13" s="10">
         <v>0.6</v>
       </c>
-      <c r="D13" s="28">
-        <v>3</v>
-      </c>
-      <c r="E13" s="28">
+      <c r="D13" s="27">
+        <v>3</v>
+      </c>
+      <c r="E13" s="27">
         <v>7</v>
       </c>
-      <c r="F13" s="29">
+      <c r="F13" s="28">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
@@ -1247,18 +1250,21 @@
       <c r="C14" s="10">
         <v>0.7</v>
       </c>
-      <c r="D14" s="28">
-        <v>3</v>
-      </c>
-      <c r="E14" s="28">
+      <c r="D14" s="27">
+        <v>3</v>
+      </c>
+      <c r="E14" s="27">
         <v>7</v>
       </c>
-      <c r="F14" s="29">
+      <c r="F14" s="28">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
       <c r="G14" s="1">
         <v>1</v>
+      </c>
+      <c r="H14" s="8" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.3">
@@ -1271,13 +1277,13 @@
       <c r="C15" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="D15" s="28">
-        <v>3</v>
-      </c>
-      <c r="E15" s="28">
+      <c r="D15" s="27">
+        <v>3</v>
+      </c>
+      <c r="E15" s="27">
         <v>7</v>
       </c>
-      <c r="F15" s="29">
+      <c r="F15" s="28">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
@@ -1295,13 +1301,13 @@
       <c r="C16" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="D16" s="28">
-        <v>3</v>
-      </c>
-      <c r="E16" s="28">
+      <c r="D16" s="27">
+        <v>3</v>
+      </c>
+      <c r="E16" s="27">
         <v>5</v>
       </c>
-      <c r="F16" s="29">
+      <c r="F16" s="28">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
@@ -1319,13 +1325,13 @@
       <c r="C17" s="10">
         <v>0.5</v>
       </c>
-      <c r="D17" s="28">
-        <v>3</v>
-      </c>
-      <c r="E17" s="28">
+      <c r="D17" s="27">
+        <v>3</v>
+      </c>
+      <c r="E17" s="27">
         <v>7</v>
       </c>
-      <c r="F17" s="29">
+      <c r="F17" s="28">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
@@ -1346,13 +1352,13 @@
       <c r="C18" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="D18" s="28">
-        <v>3</v>
-      </c>
-      <c r="E18" s="28">
+      <c r="D18" s="27">
+        <v>3</v>
+      </c>
+      <c r="E18" s="27">
         <v>4</v>
       </c>
-      <c r="F18" s="29">
+      <c r="F18" s="28">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
@@ -1370,23 +1376,23 @@
       <c r="A19" s="13" t="s">
         <v>38</v>
       </c>
-      <c r="B19" s="23" t="s">
+      <c r="B19" s="22" t="s">
         <v>39</v>
       </c>
-      <c r="C19" s="24" t="s">
-        <v>3</v>
-      </c>
-      <c r="D19" s="30">
-        <v>0</v>
-      </c>
-      <c r="E19" s="28">
-        <v>0</v>
-      </c>
-      <c r="F19" s="29">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G19" s="25">
+      <c r="C19" s="23" t="s">
+        <v>3</v>
+      </c>
+      <c r="D19" s="29">
+        <v>0</v>
+      </c>
+      <c r="E19" s="27">
+        <v>0</v>
+      </c>
+      <c r="F19" s="28">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G19" s="24">
         <v>8</v>
       </c>
       <c r="H19" s="1" t="s">
@@ -1403,13 +1409,13 @@
       <c r="C20" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="D20" s="28">
-        <v>3</v>
-      </c>
-      <c r="E20" s="28">
+      <c r="D20" s="27">
+        <v>3</v>
+      </c>
+      <c r="E20" s="27">
         <v>7</v>
       </c>
-      <c r="F20" s="29">
+      <c r="F20" s="28">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
@@ -1430,13 +1436,13 @@
       <c r="C21" s="17" t="s">
         <v>3</v>
       </c>
-      <c r="D21" s="31">
-        <v>0</v>
-      </c>
-      <c r="E21" s="28">
-        <v>0</v>
-      </c>
-      <c r="F21" s="29">
+      <c r="D21" s="30">
+        <v>0</v>
+      </c>
+      <c r="E21" s="27">
+        <v>0</v>
+      </c>
+      <c r="F21" s="28">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -1454,13 +1460,13 @@
       <c r="C22" s="20" t="s">
         <v>3</v>
       </c>
-      <c r="D22" s="32">
-        <v>0</v>
-      </c>
-      <c r="E22" s="33">
-        <v>0</v>
-      </c>
-      <c r="F22" s="34">
+      <c r="D22" s="31">
+        <v>0</v>
+      </c>
+      <c r="E22" s="32">
+        <v>0</v>
+      </c>
+      <c r="F22" s="33">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -1505,6 +1511,7 @@
     <hyperlink ref="H12" r:id="rId5" display="https://github.com/IgorRdrigues/Projeto-Java" xr:uid="{6411B9AA-E50B-479A-B839-F898EC0ECF1F}"/>
     <hyperlink ref="H17" r:id="rId6" display="https://github.com/NotKing22/Javaweb-project" xr:uid="{51423599-3084-441B-9700-DDD603589AFF}"/>
     <hyperlink ref="H4" r:id="rId7" display="https://github.com/Brunosm11/wayfit" xr:uid="{EC5ED2FC-232A-4FD2-9CA7-821BDDB52568}"/>
+    <hyperlink ref="H14" r:id="rId8" display="https://github.com/jairocket/find-your-home" xr:uid="{D876DF41-5BAC-4BC5-9AD8-A5028CC70ED8}"/>
   </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>

<commit_message>
NF java poo ... 17Jun2024
</commit_message>
<xml_diff>
--- a/03 Assessments/NOTAS AV - POO Java - 2024.1 Wyden UniRuy.xlsx
+++ b/03 Assessments/NOTAS AV - POO Java - 2024.1 Wyden UniRuy.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\YduqsArea1\16 WydenArea1 Desenvolvimento de Software Java\03 Assessments\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5F17939-3225-4C76-98B5-9D2F49E6FC2F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C333310F-1118-44FD-8C48-DA9126C41293}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{413AB662-3705-4BE9-8AD4-FDF0F3F54212}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="62">
   <si>
     <t>PBL</t>
   </si>
@@ -219,6 +219,9 @@
   </si>
   <si>
     <t>GitHub - jairocket/find-your-home: Atividade acadêmica para avaliação da disciplina Programação Orientada a Objetos com Java</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dia 12/06 - postagem https://github.com/PedroLantyer/stocker </t>
   </si>
 </sst>
 </file>
@@ -271,7 +274,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -296,6 +299,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="15">
     <border>
@@ -499,7 +508,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -575,6 +584,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hiperlink" xfId="1" builtinId="8"/>
@@ -1386,17 +1396,17 @@
         <v>0</v>
       </c>
       <c r="E19" s="27">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="F19" s="28">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="G19" s="24">
+        <v>7</v>
+      </c>
+      <c r="G19" s="35">
         <v>8</v>
       </c>
       <c r="H19" s="1" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
     </row>
     <row r="20" spans="1:15" x14ac:dyDescent="0.3">

</xml_diff>